<commit_message>
scan: seg7 2026-08-03 18:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-03.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-03.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O124"/>
+  <dimension ref="A1:O125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6965</v>
+        <v>7828</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>創新服務</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>331.0639583313744</v>
+        <v>332.9244439550691</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>77</v>
+        <v>1465</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>42.78013421095776</v>
+        <v>41.50569584763085</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>30.17400384658796</v>
+        <v>21.22023866222471</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1.071891089638085</v>
+        <v>0.5406413629080657</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.07238592381065161</v>
+        <v>-71.74035263837068</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6903</v>
+        <v>6965</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>巨漢</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>326.0352834727645</v>
+        <v>331.0639583313744</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>309.5</v>
+        <v>77</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>39.2000725958506</v>
+        <v>42.78013421095776</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>22.48295240276193</v>
+        <v>30.17400384658796</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.5631898566208265</v>
+        <v>1.071891089638085</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-7.262139082966801</v>
+        <v>-0.07238592381065161</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>7768</v>
+        <v>6903</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>巨漢</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>323.4962296557476</v>
+        <v>326.0352834727645</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>251.5</v>
+        <v>309.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>28.0924799934713</v>
+        <v>39.2000725958506</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>43.70231217434259</v>
+        <v>22.48295240276193</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.839668131205671</v>
+        <v>0.5631898566208265</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-4.351965953977281</v>
+        <v>-7.262139082966801</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6899</v>
+        <v>7768</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>321.8365663624671</v>
+        <v>323.4962296557476</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>50</v>
+        <v>251.5</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>32.61518554491678</v>
+        <v>28.0924799934713</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>27.61086536779321</v>
+        <v>43.70231217434259</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.3179029775619942</v>
+        <v>0.839668131205671</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.0199484866918497</v>
+        <v>-4.351965953977281</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2965,21 +2965,21 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>7749</v>
+        <v>6899</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>320.1562725648096</v>
+        <v>321.8365663624671</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>338</v>
+        <v>50</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>36.62758546507487</v>
+        <v>32.61518554491678</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>36.10579892996358</v>
+        <v>27.61086536779321</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.8333321949163032</v>
+        <v>0.3179029775619942</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-1.748231595975167</v>
+        <v>-0.0199484866918497</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>8044</v>
+        <v>7749</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>網家</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>318.6436466173517</v>
+        <v>320.1562725648096</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>26.2</v>
+        <v>338</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>43.9466275146699</v>
+        <v>36.62758546507487</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>19.6186074413988</v>
+        <v>36.10579892996358</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.4276195448286435</v>
+        <v>0.8333321949163032</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.0596225797547708</v>
+        <v>-1.748231595975167</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, dealer_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6937</v>
+        <v>8044</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>天虹</t>
+          <t>網家</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>317.8883673061688</v>
+        <v>318.6436466173517</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>258.5</v>
+        <v>26.2</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>46.55013471958846</v>
+        <v>43.9466275146699</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>11.71302232281533</v>
+        <v>19.6186074413988</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.46556554249201</v>
+        <v>0.4276195448286435</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.898972377326338</v>
+        <v>-0.0596225797547708</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>7822</v>
+        <v>6937</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>倍利科</t>
+          <t>天虹</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>309.6675957931512</v>
+        <v>317.8883673061688</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>778</v>
+        <v>258.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>33.85677737588765</v>
+        <v>46.55013471958846</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>27.38721194756209</v>
+        <v>11.71302232281533</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.8682757230985452</v>
+        <v>0.46556554249201</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-8.697151535081559</v>
+        <v>-1.898972377326338</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6859</v>
+        <v>7822</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>倍利科</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>304.6930940119361</v>
+        <v>309.6675957931512</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>99.2</v>
+        <v>778</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>33.05831345120998</v>
+        <v>33.85677737588765</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>30.92227103703246</v>
+        <v>27.38721194756209</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.1665325404868701</v>
+        <v>0.8682757230985452</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.114305775456545</v>
+        <v>-8.697151535081559</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>8011</v>
+        <v>6859</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>台通</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>303.228740629964</v>
+        <v>304.6930940119361</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>16.75</v>
+        <v>99.2</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>48.88644486059884</v>
+        <v>33.05831345120998</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>30.85208940903783</v>
+        <v>30.92227103703246</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>1.207674431425011</v>
+        <v>0.1665325404868701</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0325486854491701</v>
+        <v>0.114305775456545</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3283,21 +3283,21 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6865</v>
+        <v>8011</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>偉康科技</t>
+          <t>台通</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>301.3854856135182</v>
+        <v>303.228740629964</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>25.25</v>
+        <v>16.75</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>51.32554674168225</v>
+        <v>48.88644486059884</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>9.97564350170922</v>
+        <v>30.85208940903783</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.747612868882457</v>
+        <v>1.207674431425011</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0718066781756143</v>
+        <v>0.0325486854491701</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, volume_break, market_above_ma60, avoid_chase, hist_turn_positive, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>8024</v>
+        <v>6865</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>偉康科技</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>296.8935137576406</v>
+        <v>301.3854856135182</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>14</v>
+        <v>25.25</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>42.9613356705825</v>
+        <v>51.32554674168225</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>23.0276985351617</v>
+        <v>9.97564350170922</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.1908212325716205</v>
+        <v>1.747612868882457</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>1</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.3618404583162447</v>
+        <v>0.0718066781756143</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>macd_golden_cross, volume_break, market_above_ma60, avoid_chase, hist_turn_positive, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6887</v>
+        <v>8024</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>295.873295131029</v>
+        <v>296.8935137576406</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>48.07889542878456</v>
+        <v>42.9613356705825</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>14.59250468588154</v>
+        <v>23.0276985351617</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.2941835633076559</v>
+        <v>0.1908212325716205</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.1982183193398395</v>
+        <v>-0.3618404583162447</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>7717</v>
+        <v>6887</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>萊德光電-KY</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>293.2195147756665</v>
+        <v>295.873295131029</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>392.5</v>
+        <v>36</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>41.66931136350523</v>
+        <v>48.07889542878456</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.62737079698412</v>
+        <v>14.59250468588154</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4950140463631035</v>
+        <v>0.2941835633076559</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-3.087890182516574</v>
+        <v>-0.1982183193398395</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>7721</v>
+        <v>7717</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>萊德光電-KY</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>288.8318209544935</v>
+        <v>293.2195147756665</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>59.7</v>
+        <v>392.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>38.28604634324273</v>
+        <v>41.66931136350523</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>26.4120431274295</v>
+        <v>29.62737079698412</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.4508230245161341</v>
+        <v>0.4950140463631035</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.3176233939182054</v>
+        <v>-3.087890182516574</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>8034</v>
+        <v>7721</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>榮群</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>287.3358956523676</v>
+        <v>288.8318209544935</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>18.95</v>
+        <v>59.7</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>37.08975176490981</v>
+        <v>38.28604634324273</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>39.07485239353711</v>
+        <v>26.4120431274295</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.705848905925571</v>
+        <v>0.4508230245161341</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0360055575656219</v>
+        <v>-0.3176233939182054</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6855</v>
+        <v>8034</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>數泓科</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>282.2158745196872</v>
+        <v>287.3358956523676</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>117</v>
+        <v>18.95</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>51.80261117858743</v>
+        <v>37.08975176490981</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>6.421311971520948</v>
+        <v>39.07485239353711</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.1769381215929424</v>
+        <v>0.705848905925571</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>1.797697130556335</v>
+        <v>-0.0360055575656219</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>7556</v>
+        <v>6855</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>意德士</t>
+          <t>數泓科</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>280.5727735724385</v>
+        <v>282.2158745196872</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>215</v>
+        <v>117</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>38.65692407048545</v>
+        <v>51.80261117858743</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>36.92510041208624</v>
+        <v>6.421311971520948</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.3002497881682935</v>
+        <v>0.1769381215929424</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.9090023366823204</v>
+        <v>1.797697130556335</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>7728</v>
+        <v>7556</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>意德士</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>276.5838880141486</v>
+        <v>280.5727735724385</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>575</v>
+        <v>215</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>40.74158558083928</v>
+        <v>38.65692407048545</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>21.31520886077492</v>
+        <v>36.92510041208624</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.7300856579776663</v>
+        <v>0.3002497881682935</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-7.667363302600005</v>
+        <v>-0.9090023366823204</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3760,21 +3760,21 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>7744</v>
+        <v>7728</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>崴寶</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>273.4262863694171</v>
+        <v>276.5838880141486</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>401.5</v>
+        <v>575</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>39.1704922152761</v>
+        <v>40.74158558083928</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.38648039133516</v>
+        <v>21.31520886077492</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.2823959300207964</v>
+        <v>0.7300856579776663</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.467771423941205</v>
+        <v>-7.667363302600005</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3813,21 +3813,21 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>7631</v>
+        <v>7744</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>聚賢研發-創</t>
+          <t>崴寶</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>270.0952559496219</v>
+        <v>273.4262863694171</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>132.5</v>
+        <v>401.5</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>43.47369109212977</v>
+        <v>39.1704922152761</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>11.31907316584436</v>
+        <v>22.38648039133516</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.3528403561908245</v>
+        <v>0.2823959300207964</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-1.80752311344775</v>
+        <v>-2.467771423941205</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>7689</v>
+        <v>7631</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>聚賢研發-創</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>266.1986330249178</v>
+        <v>270.0952559496219</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>171</v>
+        <v>132.5</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>20.76763161329698</v>
+        <v>43.47369109212977</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>27.55683941141454</v>
+        <v>11.31907316584436</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.8198633024917795</v>
+        <v>0.3528403561908245</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-4.080354108189976</v>
+        <v>-1.80752311344775</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6936</v>
+        <v>7689</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>永鴻生技</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>261.2127543466973</v>
+        <v>266.1986330249178</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>31.85</v>
+        <v>171</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>42.55379418765989</v>
+        <v>20.76763161329698</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>14.80317418040159</v>
+        <v>27.55683941141454</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>1.0325411274244</v>
+        <v>0.8198633024917795</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.026308943363827</v>
+        <v>-4.080354108189976</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>7547</v>
+        <v>6936</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>碩網</t>
+          <t>永鴻生技</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>261.0494506204871</v>
+        <v>261.2127543466973</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>47.1</v>
+        <v>31.85</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>30.76374321615577</v>
+        <v>42.55379418765989</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>27.30931672496874</v>
+        <v>14.80317418040159</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>1.011775752976694</v>
+        <v>1.0325411274244</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.618848553645424</v>
+        <v>0.026308943363827</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6924</v>
+        <v>7547</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>榮惠-KY創</t>
+          <t>碩網</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>260.7867107875679</v>
+        <v>261.0494506204871</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>100</v>
+        <v>47.1</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>37.20310146316215</v>
+        <v>30.76374321615577</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>24.23231249903854</v>
+        <v>27.30931672496874</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>1.047564786002824</v>
+        <v>1.011775752976694</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.4461921335625396</v>
+        <v>-0.618848553645424</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6862</v>
+        <v>6924</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>榮惠-KY創</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>255.9983620026934</v>
+        <v>260.7867107875679</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>137.5</v>
+        <v>100</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>39.84730833547606</v>
+        <v>37.20310146316215</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>26.70856225306463</v>
+        <v>24.23231249903854</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.8788842430455642</v>
+        <v>1.047564786002824</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-1.961934730036198</v>
+        <v>-0.4461921335625396</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6902</v>
+        <v>6862</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>GOGOLOOK</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>254.88530132069</v>
+        <v>255.9983620026934</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>123</v>
+        <v>137.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>47.55131529426259</v>
+        <v>39.84730833547606</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>19.39061234280652</v>
+        <v>26.70856225306463</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.9734708310396371</v>
+        <v>0.8788842430455642</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.2768510191765774</v>
+        <v>-1.961934730036198</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>7799</v>
+        <v>6902</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>禾榮科</t>
+          <t>GOGOLOOK</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>253.8005787935641</v>
+        <v>254.88530132069</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>352</v>
+        <v>123</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>40.2473691273201</v>
+        <v>47.55131529426259</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>23.86653170073065</v>
+        <v>19.39061234280652</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.2110686964025499</v>
+        <v>0.9734708310396371</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-9.909104726536782</v>
+        <v>-0.2768510191765774</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>7842</v>
+        <v>7799</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>禾榮科</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>251.36227147491</v>
+        <v>253.8005787935641</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>76</v>
+        <v>352</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>43.47603549266217</v>
+        <v>40.2473691273201</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>11.5684973496196</v>
+        <v>23.86653170073065</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>4.964537635739257</v>
+        <v>0.2110686964025499</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0678736072351586</v>
+        <v>-9.909104726536782</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>7722</v>
+        <v>7842</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>LINEPAY</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>250.0807172813762</v>
+        <v>251.36227147491</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>272</v>
+        <v>76</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>38.04577241962546</v>
+        <v>43.47603549266217</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>23.759238189144</v>
+        <v>11.5684973496196</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.3618077817587529</v>
+        <v>4.964537635739257</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-4.37755102661486</v>
+        <v>-0.0678736072351586</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>8032</v>
+        <v>7722</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>LINEPAY</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>248.6116089666964</v>
+        <v>250.0807172813762</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>35.7</v>
+        <v>272</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>38.92316916795665</v>
+        <v>38.04577241962546</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>35.41684671891506</v>
+        <v>23.759238189144</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.846267921081218</v>
+        <v>0.3618077817587529</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.1522677522309634</v>
+        <v>-4.37755102661486</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4396,21 +4396,21 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6925</v>
+        <v>8032</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>意藍</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>246.4925100871231</v>
+        <v>248.6116089666964</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>51.1</v>
+        <v>35.7</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>33.98857920035296</v>
+        <v>38.92316916795665</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>18.52518076056347</v>
+        <v>35.41684671891506</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.6549846756945511</v>
+        <v>0.846267921081218</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.3211021406691543</v>
+        <v>-0.1522677522309634</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6962</v>
+        <v>6925</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>奕力-KY</t>
+          <t>意藍</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>243.8968282462817</v>
+        <v>246.4925100871231</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>31.25</v>
+        <v>51.1</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>39.24746536423403</v>
+        <v>33.98857920035296</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>28.97236029780857</v>
+        <v>18.52518076056347</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.4543504942778347</v>
+        <v>0.6549846756945511</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.24417226251165</v>
+        <v>-0.3211021406691543</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6955</v>
+        <v>6962</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>邦睿生技-創</t>
+          <t>奕力-KY</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>243.7059052813797</v>
+        <v>243.8968282462817</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0</v>
+        <v>31.25</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>18.23471488137035</v>
+        <v>39.24746536423403</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>9.994883524026942</v>
+        <v>28.97236029780857</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.0125316648316728</v>
+        <v>0.4543504942778347</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-6.490776028439575</v>
+        <v>-0.24417226251165</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6953</v>
+        <v>6955</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>邦睿生技-創</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>241.0048284312875</v>
+        <v>243.7059052813797</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>43.85008853950753</v>
+        <v>18.23471488137035</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>12.87091726325365</v>
+        <v>9.994883524026942</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.6224917751844442</v>
+        <v>0.0125316648316728</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-1.403012059558188</v>
+        <v>-6.490776028439575</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6908</v>
+        <v>6953</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>238.2547127994252</v>
+        <v>241.0048284312875</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>33.85</v>
+        <v>210</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>34.36718569265086</v>
+        <v>43.85008853950753</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>26.29575886363493</v>
+        <v>12.87091726325365</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1.871633709305552</v>
+        <v>0.6224917751844442</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.1775613188320242</v>
+        <v>-1.403012059558188</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6921</v>
+        <v>6908</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>234.4823253947584</v>
+        <v>238.2547127994252</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>60.7</v>
+        <v>33.85</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>37.38318844543166</v>
+        <v>34.36718569265086</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>30.8576212612976</v>
+        <v>26.29575886363493</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>1.502935245896646</v>
+        <v>1.871633709305552</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.3109985381349749</v>
+        <v>-0.1775613188320242</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,21 +4714,21 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>7703</v>
+        <v>6921</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>銳澤</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>234.4662808472468</v>
+        <v>234.4823253947584</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>162.5</v>
+        <v>60.7</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>34.20801790762663</v>
+        <v>37.38318844543166</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>24.48419936842311</v>
+        <v>30.8576212612976</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.9897220978715408</v>
+        <v>1.502935245896646</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-2.835400057636344</v>
+        <v>-0.3109985381349749</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>7818</v>
+        <v>7703</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>銳澤</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>234.3456245291409</v>
+        <v>234.4662808472468</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>63.2</v>
+        <v>162.5</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>28.46340762165829</v>
+        <v>34.20801790762663</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>28.21366702498442</v>
+        <v>24.48419936842311</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.447646131584809</v>
+        <v>0.9897220978715408</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.4930147718459704</v>
+        <v>-2.835400057636344</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4820,21 +4820,21 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>7780</v>
+        <v>7818</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>大研生醫*</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>233.7630187198826</v>
+        <v>234.3456245291409</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>16.8</v>
+        <v>63.2</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>34.0842332050025</v>
+        <v>28.46340762165829</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>31.70443415803321</v>
+        <v>28.21366702498442</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.4537381203706478</v>
+        <v>0.447646131584809</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.0537797956302201</v>
+        <v>-0.4930147718459704</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6869</v>
+        <v>7780</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>大研生醫*</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>230.5131587117744</v>
+        <v>233.7630187198825</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>65.90000000000001</v>
+        <v>16.8</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>37.29266998631144</v>
+        <v>34.0842332050025</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>24.15326011420807</v>
+        <v>31.70443415803321</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.7188601615845414</v>
+        <v>0.4537381203706478</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.1106820770621714</v>
+        <v>-0.0537797956302201</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4926,21 +4926,21 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>7827</v>
+        <v>6869</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>漢康-KY創</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>228.5825844055472</v>
+        <v>230.5131587117744</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>150.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.40278950585339</v>
+        <v>37.29266998631144</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>20.00632470837925</v>
+        <v>24.15326011420807</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5704832731336438</v>
+        <v>0.7188601615845414</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-1.514923771283343</v>
+        <v>0.1106820770621714</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>7732</v>
+        <v>7827</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>金興精密</t>
+          <t>漢康-KY創</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>224.2448383381301</v>
+        <v>228.5825844055472</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>35.55</v>
+        <v>150.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>51.60627045753562</v>
+        <v>47.40278950585339</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>4.883700596313997</v>
+        <v>20.00632470837925</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.3727771047080054</v>
+        <v>0.5704832731336438</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.1035551884630919</v>
+        <v>-1.514923771283343</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6906</v>
+        <v>7732</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>金興精密</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>221.7028248066839</v>
+        <v>224.2448383381301</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>68.59999999999999</v>
+        <v>35.55</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>29.53087521573144</v>
+        <v>51.60627045753562</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>32.78941499629193</v>
+        <v>4.883700596313997</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.45763641559198</v>
+        <v>0.3727771047080054</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.1447370001804628</v>
+        <v>-0.1035551884630919</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>7791</v>
+        <v>6906</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>219.1089664900564</v>
+        <v>221.7028248066839</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>59.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>28.53020833736161</v>
+        <v>29.53087521573144</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>22.42271347965936</v>
+        <v>32.78941499629193</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.8648503216176593</v>
+        <v>0.45763641559198</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.2708097796983799</v>
+        <v>-0.1447370001804628</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5138,21 +5138,21 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>7730</v>
+        <v>7791</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>218.7884325577721</v>
+        <v>219.1089664900564</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>152</v>
+        <v>59.5</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>38.51558970033693</v>
+        <v>28.53020833736161</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>26.14853480863429</v>
+        <v>22.42271347965936</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5632537178532274</v>
+        <v>0.8648503216176593</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-2.135948166552579</v>
+        <v>-0.2708097796983799</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6983</v>
+        <v>7730</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>華洋精機</t>
+          <t>暉盛-創</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>216.3892843060379</v>
+        <v>218.7884325577721</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>303</v>
+        <v>152</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>36.57850621498733</v>
+        <v>38.51558970033693</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>12.98434808215518</v>
+        <v>26.14853480863429</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.5560143573178626</v>
+        <v>0.5632537178532274</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-2.90566276332941</v>
+        <v>-2.135948166552579</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>7738</v>
+        <v>6983</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>東聯互動</t>
+          <t>華洋精機</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>212.9424663289402</v>
+        <v>216.3892843060379</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>166</v>
+        <v>303</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>45.74983014867541</v>
+        <v>36.57850621498733</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>27.15576298203587</v>
+        <v>12.98434808215518</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.3300428870207762</v>
+        <v>0.5560143573178626</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1789471818274843</v>
+        <v>-2.90566276332941</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>7820</v>
+        <v>7738</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>立盈</t>
+          <t>東聯互動</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>208.5191693044854</v>
+        <v>212.9424663289402</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>103</v>
+        <v>166</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>37.78580607976613</v>
+        <v>45.74983014867541</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>22.35265155433076</v>
+        <v>27.15576298203587</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.1902429007275287</v>
+        <v>0.3300428870207762</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.6769006809541134</v>
+        <v>-0.1789471818274843</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6923</v>
+        <v>7820</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>立盈</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>205.9323270004896</v>
+        <v>208.5191693044854</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>75.59999999999999</v>
+        <v>103</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>45.48592399842367</v>
+        <v>37.78580607976613</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>11.71957274810677</v>
+        <v>22.35265155433076</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.369108306299921</v>
+        <v>0.1902429007275287</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.1972167144030206</v>
+        <v>-0.6769006809541134</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6910</v>
+        <v>6923</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>德鴻</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>205.7783482484212</v>
+        <v>205.9323270004896</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>24.4</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>35.4345355922532</v>
+        <v>45.48592399842367</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>29.80624163695926</v>
+        <v>11.71957274810677</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.901737531009984</v>
+        <v>0.369108306299921</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.0210117579200269</v>
+        <v>-0.1972167144030206</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6933</v>
+        <v>6910</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>AMAX-KY</t>
+          <t>德鴻</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>201.741149416183</v>
+        <v>205.7783482484212</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>154</v>
+        <v>24.4</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>48.66637053409032</v>
+        <v>35.4345355922532</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.83191605444226</v>
+        <v>29.80624163695926</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>1.107509315547642</v>
+        <v>0.901737531009984</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-1.582738633294978</v>
+        <v>-0.0210117579200269</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6934</v>
+        <v>6933</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>心誠鎂</t>
+          <t>AMAX-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>200.2622638546855</v>
+        <v>201.741149416183</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>76.59999999999999</v>
+        <v>154</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>52.89888314895735</v>
+        <v>48.66637053409032</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>17.80539980275046</v>
+        <v>14.83191605444226</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.0906457646807594</v>
+        <v>1.107509315547642</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.5992204432878776</v>
+        <v>-1.582738633294978</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6916</v>
+        <v>6934</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>心誠鎂</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>200.0648720402208</v>
+        <v>200.2622638546855</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>18.05</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>40.55314274237416</v>
+        <v>52.89888314895735</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>17.58025378372151</v>
+        <v>17.80539980275046</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.351391484570176</v>
+        <v>0.0906457646807594</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.2501127247279687</v>
+        <v>-0.5992204432878776</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>7402</v>
+        <v>6916</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>194.8056218156132</v>
+        <v>200.0648720402208</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>101</v>
+        <v>18.05</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.07800515750544</v>
+        <v>40.55314274237416</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>23.23009683628903</v>
+        <v>17.58025378372151</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.1302995285501577</v>
+        <v>0.351391484570176</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-3.209333939835862</v>
+        <v>-0.2501127247279687</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6967</v>
+        <v>7402</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>188.1952676873717</v>
+        <v>194.8056218156132</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>69.09999999999999</v>
+        <v>101</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>43.54838722955843</v>
+        <v>42.07800515750544</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.71157640782386</v>
+        <v>23.23009683628903</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.1490673676700962</v>
+        <v>0.1302995285501577</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.8375878106592313</v>
+        <v>-3.209333939835862</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6971</v>
+        <v>6967</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>187.1538573075597</v>
+        <v>188.1952676873717</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>25.9</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>35.47348947278054</v>
+        <v>43.54838722955843</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>15.58617719088696</v>
+        <v>16.71157640782386</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.8320780855122517</v>
+        <v>0.1490673676700962</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1325625649068154</v>
+        <v>-0.8375878106592313</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>7803</v>
+        <v>6971</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>雲象科技-創</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>186.1884131298962</v>
+        <v>187.1538573075597</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>19.5</v>
+        <v>25.9</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>32.84824209973047</v>
+        <v>35.47348947278054</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>25.12704751467234</v>
+        <v>15.58617719088696</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.4680418225364626</v>
+        <v>0.8320780855122517</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.1578261792063622</v>
+        <v>-0.1325625649068154</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6918</v>
+        <v>7803</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>愛派司</t>
+          <t>雲象科技-創</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>184.6157034835362</v>
+        <v>186.1884131298962</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>70.40000000000001</v>
+        <v>19.5</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.00502880197797</v>
+        <v>32.84824209973047</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>15.21904686145772</v>
+        <v>25.12704751467234</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.783115023111516</v>
+        <v>0.4680418225364626</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2401744663131959</v>
+        <v>-0.1578261792063622</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6913</v>
+        <v>6918</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>鴻呈</t>
+          <t>愛派司</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>181.5657167574307</v>
+        <v>184.6157034835362</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>124.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>52.1249871088126</v>
+        <v>41.00502880197797</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>13.6979309498782</v>
+        <v>15.21904686145772</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.713525227825176</v>
+        <v>1.783115023111516</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0612958430634806</v>
+        <v>-0.2401744663131959</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6854</v>
+        <v>6913</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>鴻呈</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>181.4647380645115</v>
+        <v>181.5657167574307</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>91.7</v>
+        <v>124.5</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>31.95822406625564</v>
+        <v>52.1249871088126</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>46.10721296065853</v>
+        <v>13.6979309498782</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.4525865603805388</v>
+        <v>0.713525227825176</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.3258985712596356</v>
+        <v>-0.0612958430634806</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6894</v>
+        <v>6854</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>177.3091099863314</v>
+        <v>181.4647380645115</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>332</v>
+        <v>91.7</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>48.33062165040581</v>
+        <v>31.95822406625564</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>19.17832061470708</v>
+        <v>46.10721296065853</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.9937063117439192</v>
+        <v>0.4525865603805388</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.459500911636038</v>
+        <v>-0.3258985712596356</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6890</v>
+        <v>6894</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>176.1556196681638</v>
+        <v>177.3091099863314</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>166</v>
+        <v>332</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>37.07444549384746</v>
+        <v>48.33062165040581</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.28625900762501</v>
+        <v>19.17832061470708</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.6387325346656052</v>
+        <v>0.9937063117439192</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.1835661994801576</v>
+        <v>-0.459500911636038</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>7823</v>
+        <v>6890</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>奧義賽博-KY創</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>169.5675418700106</v>
+        <v>176.1556196681638</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>78.3</v>
+        <v>166</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>39.41421350623074</v>
+        <v>37.07444549384746</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>20.69202632507284</v>
+        <v>16.28625900762501</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.7610231780087465</v>
+        <v>0.6387325346656052</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.3990365208182505</v>
+        <v>-0.1835661994801576</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6909</v>
+        <v>7823</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>奧義賽博-KY創</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>161.0333236536362</v>
+        <v>169.5675418700106</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>40.05</v>
+        <v>78.3</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>35.39334875144431</v>
+        <v>39.41421350623074</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>30.86772213613765</v>
+        <v>20.69202632507284</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.5196182867799369</v>
+        <v>0.7610231780087465</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.487096605375565</v>
+        <v>-0.3990365208182505</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>7736</v>
+        <v>6909</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>158.0692433451451</v>
+        <v>161.0333236536362</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>70.40000000000001</v>
+        <v>40.05</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>45.91197388168772</v>
+        <v>35.39334875144431</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>24.37687593140397</v>
+        <v>30.86772213613765</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.7069243345145065</v>
+        <v>0.5196182867799369</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.08904051372468059</v>
+        <v>-0.487096605375565</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6251,21 +6251,21 @@
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6873</v>
+        <v>7736</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>虎山</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>156.6454995748129</v>
+        <v>158.0692433451451</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>77.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>39.33581210808028</v>
+        <v>45.91197388168772</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>16.33767100242729</v>
+        <v>24.37687593140397</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.4750110874542387</v>
+        <v>0.7069243345145065</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.9277799455297338</v>
+        <v>0.08904051372468059</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6895</v>
+        <v>6873</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>156.2031945071398</v>
+        <v>156.6454995748129</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>117</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>32.44831614128947</v>
+        <v>39.33581210808028</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>31.69651782563198</v>
+        <v>16.33767100242729</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.5006267599882105</v>
+        <v>0.4750110874542387</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0136753906868456</v>
+        <v>-0.9277799455297338</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6928</v>
+        <v>6895</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>152.8497908420817</v>
+        <v>156.2031945071398</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>48.6</v>
+        <v>117</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.10875844098362</v>
+        <v>32.44831614128947</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>21.94478059502445</v>
+        <v>31.69651782563198</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.1268324513998847</v>
+        <v>0.5006267599882105</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.9157028894225976</v>
+        <v>-0.0136753906868456</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6410,21 +6410,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>7810</v>
+        <v>6928</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>捷創科技</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>152.5029891580187</v>
+        <v>152.8497908420817</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>180.5</v>
+        <v>48.6</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>35.60605228110646</v>
+        <v>46.10875844098362</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>17.07826303339925</v>
+        <v>21.94478059502445</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.7229300008101758</v>
+        <v>0.1268324513998847</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-1.661511098663743</v>
+        <v>-0.9157028894225976</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6997</v>
+        <v>7810</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>博弘</t>
+          <t>捷創科技</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>149.6988449525005</v>
+        <v>152.5029891580187</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>72</v>
+        <v>180.5</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>53.09517990848064</v>
+        <v>35.60605228110646</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>12.79414808777058</v>
+        <v>17.07826303339925</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.8628491184272117</v>
+        <v>0.7229300008101758</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-1.997493643435732</v>
+        <v>-1.661511098663743</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6931</v>
+        <v>6997</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>青松健康</t>
+          <t>博弘</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>139.2468840995494</v>
+        <v>149.6988449525005</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>37.95</v>
+        <v>72</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.44328631233385</v>
+        <v>53.09517990848064</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>16.92468747523838</v>
+        <v>12.79414808777058</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.245758077552578</v>
+        <v>0.8628491184272117</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1293649543411771</v>
+        <v>-1.997493643435732</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>7765</v>
+        <v>6931</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>青松健康</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>134.3413583732514</v>
+        <v>139.2468840995494</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>222.5</v>
+        <v>37.95</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.34068398332218</v>
+        <v>40.44328631233385</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>13.60466309830841</v>
+        <v>16.92468747523838</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.9856224231957994</v>
+        <v>1.245758077552578</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.4483366250274407</v>
+        <v>-0.1293649543411771</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6622,21 +6622,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>7786</v>
+        <v>7765</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>東方風能</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>132.8731629558942</v>
+        <v>134.3413583732514</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>125</v>
+        <v>222.5</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>46.77278650189889</v>
+        <v>43.34068398332218</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>13.78804094469301</v>
+        <v>13.60466309830841</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.3968234846477062</v>
+        <v>0.9856224231957994</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.6701470158308914</v>
+        <v>0.4483366250274407</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6675,21 +6675,21 @@
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>7760</v>
+        <v>7786</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>東方風能</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>130.940946969789</v>
+        <v>132.8731629558942</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>33.8</v>
+        <v>125</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>45.42323625903432</v>
+        <v>46.77278650189889</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>19.67375291715303</v>
+        <v>13.78804094469301</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>1.521255086362639</v>
+        <v>0.3968234846477062</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1568350443390781</v>
+        <v>-0.6701470158308914</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6885</v>
+        <v>7760</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>120.1837565965366</v>
+        <v>130.940946969789</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>21.1</v>
+        <v>33.8</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>47.54729741332899</v>
+        <v>45.42323625903432</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>10.40854765936272</v>
+        <v>19.67375291715303</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.3790401040760165</v>
+        <v>1.521255086362639</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.0432249430827432</v>
+        <v>-0.1568350443390781</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>7705</v>
+        <v>6885</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>三商餐飲</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>111.5675636451648</v>
+        <v>120.1837565965366</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>30.2</v>
+        <v>21.1</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>41.86026814678132</v>
+        <v>47.54729741332899</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.20157180375306</v>
+        <v>10.40854765936272</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.2931039524750489</v>
+        <v>0.3790401040760165</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0084519475504928</v>
+        <v>0.0432249430827432</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>7753</v>
+        <v>7705</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>三商餐飲</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>110.6082486615187</v>
+        <v>111.5675636451648</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>38.45</v>
+        <v>30.2</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>41.63693680905475</v>
+        <v>41.86026814678132</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>17.19865445799099</v>
+        <v>15.20157180375306</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.6010953809294588</v>
+        <v>0.2931039524750489</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.3326662724626537</v>
+        <v>-0.0084519475504928</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6887,21 +6887,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>8038</v>
+        <v>7753</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>長園科</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>77.71987490967729</v>
+        <v>110.6082486615187</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>31.45</v>
+        <v>38.45</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,16 +6912,16 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>30.87674895416467</v>
+        <v>41.63693680905475</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>19.2852788020834</v>
+        <v>17.19865445799099</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.2287416382611054</v>
+        <v>0.6010953809294588</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.7011206708001356</v>
+        <v>-0.3326662724626537</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6988</v>
+        <v>8038</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>威力暘-創</t>
+          <t>長園科</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>32.14188845187701</v>
+        <v>77.71987490967729</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>11.95</v>
+        <v>31.45</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>48.73261879457369</v>
+        <v>30.87674895416467</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.85108857169023</v>
+        <v>19.2852788020834</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.9845333423337524</v>
+        <v>0.2287416382611054</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,62 +6983,115 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0661232452963291</v>
+        <v>-0.7011206708001356</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
+        <v>6988</v>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>威力暘-創</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>32.14188845187701</v>
+      </c>
+      <c r="E124" s="2" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H124" s="2" t="n">
+        <v>48.73261879457369</v>
+      </c>
+      <c r="I124" s="2" t="n">
+        <v>13.85108857169023</v>
+      </c>
+      <c r="J124" s="2" t="n">
+        <v>0.9845333423337524</v>
+      </c>
+      <c r="K124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N124" s="2" t="n">
+        <v>0.0661232452963291</v>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="B124" s="2" t="inlineStr">
+      <c r="B125" s="2" t="inlineStr">
         <is>
           <t>君曜</t>
         </is>
       </c>
-      <c r="C124" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D124" s="2" t="n">
+      <c r="C125" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D125" s="2" t="n">
         <v>-13.63143717795565</v>
       </c>
-      <c r="E124" s="2" t="n">
+      <c r="E125" s="2" t="n">
         <v>39.8</v>
       </c>
-      <c r="F124" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="G124" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H124" s="2" t="n">
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H125" s="2" t="n">
         <v>50.35157927622254</v>
       </c>
-      <c r="I124" s="2" t="n">
+      <c r="I125" s="2" t="n">
         <v>10.79172389250918</v>
       </c>
-      <c r="J124" s="2" t="n">
+      <c r="J125" s="2" t="n">
         <v>0.2592955113953953</v>
       </c>
-      <c r="K124" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L124" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M124" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N124" s="2" t="n">
+      <c r="K125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N125" s="2" t="n">
         <v>0.3294355447212704</v>
       </c>
-      <c r="O124" s="2" t="inlineStr">
+      <c r="O125" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60</t>
         </is>

</xml_diff>